<commit_message>
Add Instructions sheet to upload template and skip it during parsing
- Added Instructions sheet as the first tab in the Excel upload template
  with step-by-step guidance on filling out data and uploading
- Updated create_upload_template.py to generate the Instructions sheet
- Updated excel_parser.py fallback logic to skip the Instructions sheet
  when looking for data sheets by index

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -7,8 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,13 +21,44 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="22"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00025A9A"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00444444"/>
+      <sz val="13"/>
     </font>
     <font>
       <b val="1"/>
@@ -44,12 +76,24 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00025A9A"/>
+        <bgColor rgb="00025A9A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
+        <bgColor rgb="00E8F4FD"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -88,28 +132,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -478,6 +551,325 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00025A9A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="55" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>BPC1 Upload Template — Instructions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="10" customHeight="1"/>
+    <row r="3" ht="40" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Step 1: Fill Out the Template</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Open the "Income Statement" and "Balance Sheet" tabs in this workbook.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Enter the dollar amounts for each line item in the Amount column (Column C). Each line item matches what you see on the dashboard's Income Statement and Balance Sheet pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Enter raw numbers only — no dollar signs ($), commas, or other formatting. For example, enter 150000 not $150,000.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Enter negative values with a minus sign (e.g., -5000 for accumulated depreciation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Enter 0 for any line item that does not apply to your company. Do not leave cells blank.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="42" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Do NOT modify the line item names in Column A or the descriptions in Column B. The system uses these names to match your data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>7.</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Do NOT fill in any rows labeled as totals (e.g., Total Revenue, Total Assets). These are calculated automatically by the dashboard.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="10" customHeight="1"/>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Step 2: Upload Your Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>1.</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Log in to the BPC1 Dashboard and navigate to the Upload page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2.</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>At the top of the page, select your company name from the dropdown.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>3.</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Select the correct reporting period — choose whether this is a Full Year or Mid Year report, and select the correct year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>4.</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>On the sidebar of the upload page, you will find an option to upload this Excel file. Click it and select this file.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>5.</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>The system will parse your data and show you a preview. Review it carefully before submitting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>6.</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Click the Submit button to upload your data. Once submitted, your data will be in "Submitted" status until an admin publishes it to the dashboard.</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="10" customHeight="1"/>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Important Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="45" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Make sure you select the correct company and period before uploading — the system will save data under whichever company and period you have selected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>This Instructions sheet is ignored during upload. Only the Income Statement and Balance Sheet sheets are processed.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23" ht="45" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>If you see warnings after upload about unmatched line items, check that the line item names in your file have not been modified.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <mergeCells count="20">
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B15:H15"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="B22:H22"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B21:H21"/>
+    <mergeCell ref="B23:H23"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B13:H13"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="B10:H10"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -490,751 +882,751 @@
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Income Statement Data Entry</t>
         </is>
       </c>
-      <c r="C1" s="2" t="n"/>
+      <c r="C1" s="13" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>12/31/25</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>REVENUE</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="13" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Intra State HHG</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Transportation revenues generated under an intrastate tariff</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n"/>
+      <c r="C4" s="19" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Local HHG</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Revenues defined by an intrastate tariff as local</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n"/>
+      <c r="C5" s="19" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Inter State HHG</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Transportation revenues generated under an interstate tariff</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n"/>
+      <c r="C6" s="19" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Office &amp; Industrial</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>All local commercial revenue except HHG</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n"/>
+      <c r="C7" s="19" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Warehouse (Non-commercial)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>All permanent and SIT revenue</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n"/>
+      <c r="C8" s="19" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Warehouse Handling (Non-commercial)</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
-      <c r="C9" s="8" t="n"/>
+      <c r="B9" s="18" t="inlineStr"/>
+      <c r="C9" s="19" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>International</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>All international revenue including pickup, packing, crating, delivery</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n"/>
+      <c r="C10" s="19" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Packing &amp; Unpacking</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>All revenue for packing, unpacking and container revenue</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n"/>
+      <c r="C11" s="19" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Booking &amp; Royalties</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>Sales booking revenue and Operating Authority royalties</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n"/>
+      <c r="C12" s="19" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Special Products</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>All special product revenue and HVP transportation</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n"/>
+      <c r="C13" s="19" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Records Storage</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>All records storage revenue</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n"/>
+      <c r="C14" s="19" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Military DPM Contracts</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Revenues from Direct Procurement Method military contracts</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n"/>
+      <c r="C15" s="19" t="n"/>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Distribution</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="18" t="inlineStr">
         <is>
           <t>All distribution revenue</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n"/>
+      <c r="C16" s="19" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Hotel Deliveries</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>All revenues from hotel deliveries</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n"/>
+      <c r="C17" s="19" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Other Revenue</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>Any misc. operational revenue not listed elsewhere</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
+      <c r="C18" s="19" t="n"/>
     </row>
     <row r="19" ht="8" customHeight="1">
-      <c r="C19" s="2" t="n"/>
+      <c r="C19" s="13" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>DIRECT EXPENSES (COST OF REVENUE)</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n"/>
+      <c r="C20" s="13" t="n"/>
     </row>
     <row r="21" ht="30" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Direct Wages</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="18" t="inlineStr">
         <is>
           <t>Salaries, wages, and bonuses paid to operations personnel</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n"/>
+      <c r="C21" s="19" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Vehicle Operating Expense</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>Repairs, fuel, license, registration, tires, permits for revenue equipment</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
+      <c r="C22" s="19" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Packing/Warehouse Supplies</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="B23" s="18" t="inlineStr">
         <is>
           <t>Moving and packing supplies</t>
         </is>
       </c>
-      <c r="C23" s="8" t="n"/>
+      <c r="C23" s="19" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>OO Exp Intra State</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Payments to owner operators for intrastate jobs</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
+      <c r="C24" s="19" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>OO Inter State</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Payments to owner operators for interstate jobs</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
+      <c r="C25" s="19" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>OO O&amp;I</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>Payments to owner operators for office &amp; industrial jobs</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
+      <c r="C26" s="19" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>OO Packing</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>Payments to owner operators for packing jobs</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
+      <c r="C27" s="19" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>OO Other</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Payments to owner operators for other job types</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
+      <c r="C28" s="19" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Claims</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="18" t="inlineStr">
         <is>
           <t>All operational claims</t>
         </is>
       </c>
-      <c r="C29" s="8" t="n"/>
+      <c r="C29" s="19" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="6" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Other Trans Exp</t>
         </is>
       </c>
-      <c r="B30" s="7" t="inlineStr">
+      <c r="B30" s="18" t="inlineStr">
         <is>
           <t>Trip expense, deadhead miles, agent fees, freight, BIPD</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n"/>
+      <c r="C30" s="19" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="18" t="inlineStr">
         <is>
           <t>Depreciation on assets (excluding buildings)</t>
         </is>
       </c>
-      <c r="C31" s="8" t="n"/>
+      <c r="C31" s="19" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Lease Expense Rev Equip</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>All lease expense on revenue equipment</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
+      <c r="C32" s="19" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Actual or estimated fair market rent</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n"/>
+      <c r="C33" s="19" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Other Direct Expenses</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>Credit card fees and other direct expenses not otherwise classified</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n"/>
+      <c r="C34" s="19" t="n"/>
     </row>
     <row r="35" ht="8" customHeight="1">
-      <c r="C35" s="2" t="n"/>
+      <c r="C35" s="13" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" s="16" t="inlineStr">
         <is>
           <t>OPERATING EXPENSES</t>
         </is>
       </c>
-      <c r="C36" s="2" t="n"/>
+      <c r="C36" s="13" t="n"/>
     </row>
     <row r="37" ht="30" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Advertising/Marketing</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="18" t="inlineStr">
         <is>
           <t>Advertising, brochures, yellow pages, promotional items</t>
         </is>
       </c>
-      <c r="C37" s="8" t="n"/>
+      <c r="C37" s="19" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Bad Debts</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>Uncollectible accounts receivable written off</t>
         </is>
       </c>
-      <c r="C38" s="8" t="n"/>
+      <c r="C38" s="19" t="n"/>
     </row>
     <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Sales Commissions</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
+      <c r="B39" s="18" t="inlineStr">
         <is>
           <t>Salaries, commissions, and draws for sales people</t>
         </is>
       </c>
-      <c r="C39" s="8" t="n"/>
+      <c r="C39" s="19" t="n"/>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="6" t="inlineStr">
+      <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Contributions</t>
         </is>
       </c>
-      <c r="B40" s="7" t="inlineStr"/>
-      <c r="C40" s="8" t="n"/>
+      <c r="B40" s="18" t="inlineStr"/>
+      <c r="C40" s="19" t="n"/>
     </row>
     <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="6" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Computer Support</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
+      <c r="B41" s="18" t="inlineStr">
         <is>
           <t>IT expenses, software licensing, satellite tracking</t>
         </is>
       </c>
-      <c r="C41" s="8" t="n"/>
+      <c r="C41" s="19" t="n"/>
     </row>
     <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="6" t="inlineStr">
+      <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
-      <c r="B42" s="7" t="inlineStr"/>
-      <c r="C42" s="8" t="n"/>
+      <c r="B42" s="18" t="inlineStr"/>
+      <c r="C42" s="19" t="n"/>
     </row>
     <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>PR Taxes &amp; Benefits</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="18" t="inlineStr">
         <is>
           <t>Payroll taxes, health insurance, drug testing, DOT physicals, training</t>
         </is>
       </c>
-      <c r="C43" s="8" t="n"/>
+      <c r="C43" s="19" t="n"/>
     </row>
     <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Equipment Leases Office Equip</t>
         </is>
       </c>
-      <c r="B44" s="7" t="inlineStr"/>
-      <c r="C44" s="8" t="n"/>
+      <c r="B44" s="18" t="inlineStr"/>
+      <c r="C44" s="19" t="n"/>
     </row>
     <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="6" t="inlineStr">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Workman's Comp Insurance</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr"/>
-      <c r="C45" s="8" t="n"/>
+      <c r="B45" s="18" t="inlineStr"/>
+      <c r="C45" s="19" t="n"/>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="6" t="inlineStr">
+      <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
-      <c r="B46" s="7" t="inlineStr">
+      <c r="B46" s="18" t="inlineStr">
         <is>
           <t>Cargo, fleet, general liability insurance</t>
         </is>
       </c>
-      <c r="C46" s="8" t="n"/>
+      <c r="C46" s="19" t="n"/>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="6" t="inlineStr">
+      <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Legal &amp; Accounting</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="B47" s="18" t="inlineStr">
         <is>
           <t>Legal and accounting work, tax return preparation</t>
         </is>
       </c>
-      <c r="C47" s="8" t="n"/>
+      <c r="C47" s="19" t="n"/>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="6" t="inlineStr">
+      <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Office Expense</t>
         </is>
       </c>
-      <c r="B48" s="7" t="inlineStr">
+      <c r="B48" s="18" t="inlineStr">
         <is>
           <t>Office &amp; printer supplies, printed forms, coffee, janitorial</t>
         </is>
       </c>
-      <c r="C48" s="8" t="n"/>
+      <c r="C48" s="19" t="n"/>
     </row>
     <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="6" t="inlineStr">
+      <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Other Admin</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr"/>
-      <c r="C49" s="8" t="n"/>
+      <c r="B49" s="18" t="inlineStr"/>
+      <c r="C49" s="19" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="6" t="inlineStr">
+      <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Pension/Profit Sharing/401k</t>
         </is>
       </c>
-      <c r="B50" s="7" t="inlineStr"/>
-      <c r="C50" s="8" t="n"/>
+      <c r="B50" s="18" t="inlineStr"/>
+      <c r="C50" s="19" t="n"/>
     </row>
     <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Professional Fees</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
+      <c r="B51" s="18" t="inlineStr">
         <is>
           <t>Consultants, detectives, non-trade professionals</t>
         </is>
       </c>
-      <c r="C51" s="8" t="n"/>
+      <c r="C51" s="19" t="n"/>
     </row>
     <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B52" s="7" t="inlineStr"/>
-      <c r="C52" s="8" t="n"/>
+      <c r="B52" s="18" t="inlineStr"/>
+      <c r="C52" s="19" t="n"/>
     </row>
     <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Salaries Admin</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
+      <c r="B53" s="18" t="inlineStr">
         <is>
           <t>All non-operations salaries (admin, office, dispatch, sales support)</t>
         </is>
       </c>
-      <c r="C53" s="8" t="n"/>
+      <c r="C53" s="19" t="n"/>
     </row>
     <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="17" t="inlineStr">
         <is>
           <t>Taxes &amp; Licenses</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="B54" s="18" t="inlineStr">
         <is>
           <t>All taxes and licenses not related to vehicles or income</t>
         </is>
       </c>
-      <c r="C54" s="8" t="n"/>
+      <c r="C54" s="19" t="n"/>
     </row>
     <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="6" t="inlineStr">
+      <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Tel/Fax/Utilities/Internet</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
+      <c r="B55" s="18" t="inlineStr">
         <is>
           <t>All communication and utility expenses</t>
         </is>
       </c>
-      <c r="C55" s="8" t="n"/>
+      <c r="C55" s="19" t="n"/>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="6" t="inlineStr">
+      <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Travel &amp; Entertainment</t>
         </is>
       </c>
-      <c r="B56" s="7" t="inlineStr">
+      <c r="B56" s="18" t="inlineStr">
         <is>
           <t>Admin/sales related transportation, meals, lodging</t>
         </is>
       </c>
-      <c r="C56" s="8" t="n"/>
+      <c r="C56" s="19" t="n"/>
     </row>
     <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Vehicle Expense Admin</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr"/>
-      <c r="C57" s="8" t="n"/>
+      <c r="B57" s="18" t="inlineStr"/>
+      <c r="C57" s="19" t="n"/>
     </row>
     <row r="58" ht="8" customHeight="1">
-      <c r="C58" s="2" t="n"/>
+      <c r="C58" s="13" t="n"/>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="5" t="inlineStr">
+      <c r="A59" s="16" t="inlineStr">
         <is>
           <t>OTHER INCOME/EXPENSES</t>
         </is>
       </c>
-      <c r="C59" s="2" t="n"/>
+      <c r="C59" s="13" t="n"/>
     </row>
     <row r="60" ht="30" customHeight="1">
-      <c r="A60" s="6" t="inlineStr">
+      <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Other Income</t>
         </is>
       </c>
-      <c r="B60" s="7" t="inlineStr">
+      <c r="B60" s="18" t="inlineStr">
         <is>
           <t>Interest income, gain on sale of asset, litigation income</t>
         </is>
       </c>
-      <c r="C60" s="8" t="n"/>
+      <c r="C60" s="19" t="n"/>
     </row>
     <row r="61" ht="30" customHeight="1">
-      <c r="A61" s="6" t="inlineStr">
+      <c r="A61" s="17" t="inlineStr">
         <is>
           <t>CEO Comp</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B61" s="18" t="inlineStr">
         <is>
           <t>All salaries, bonuses or perks paid to CEO (enter as negative)</t>
         </is>
       </c>
-      <c r="C61" s="8" t="n"/>
+      <c r="C61" s="19" t="n"/>
     </row>
     <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>Other Expense</t>
         </is>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="B62" s="18" t="inlineStr">
         <is>
           <t>Loss on sale of asset, research of new business lines (enter as negative)</t>
         </is>
       </c>
-      <c r="C62" s="8" t="n"/>
+      <c r="C62" s="19" t="n"/>
     </row>
     <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="6" t="inlineStr">
+      <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Interest Expense</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr">
+      <c r="B63" s="18" t="inlineStr">
         <is>
           <t>All interest paid on interest bearing debt (enter as negative)</t>
         </is>
       </c>
-      <c r="C63" s="8" t="n"/>
+      <c r="C63" s="19" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="5">
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A59:C59"/>
     <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A59:C59"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1249,420 +1641,420 @@
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Balance Sheet Data Entry</t>
         </is>
       </c>
-      <c r="C1" s="2" t="n"/>
+      <c r="C1" s="13" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Line Item</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>12/31/25</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>CURRENT ASSETS</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
+      <c r="C3" s="13" t="n"/>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Cash &amp; Cash Equivalents</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>All cash and money market type investments</t>
         </is>
       </c>
-      <c r="C4" s="8" t="n"/>
+      <c r="C4" s="19" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Receivable</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="18" t="inlineStr">
         <is>
           <t>Receivables generated from customers in the course of business</t>
         </is>
       </c>
-      <c r="C5" s="8" t="n"/>
+      <c r="C5" s="19" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Receivables</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Amount owed by Van Line (if positive) or owed to Van Line (if negative)</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n"/>
+      <c r="C6" s="19" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Other Receivables</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Amounts owed by drivers, employees, etc.</t>
         </is>
       </c>
-      <c r="C7" s="8" t="n"/>
+      <c r="C7" s="19" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Prepaid Expenses</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Any prepaid expenses</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n"/>
+      <c r="C8" s="19" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Related Company Receivables</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>All receivables owing from related companies</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n"/>
+      <c r="C9" s="19" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Owner Receivables</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="18" t="inlineStr">
         <is>
           <t>All receivables owing from owners</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n"/>
+      <c r="C10" s="19" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Other Current Assets</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>Packing supplies, investments not included in cash, etc.</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n"/>
+      <c r="C11" s="19" t="n"/>
     </row>
     <row r="12" ht="8" customHeight="1">
-      <c r="C12" s="2" t="n"/>
+      <c r="C12" s="13" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>FIXED ASSETS</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n"/>
+      <c r="C13" s="13" t="n"/>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Gross Fixed Assets</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>All equipment, land, buildings, leasehold improvements, furniture and fixtures</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n"/>
+      <c r="C14" s="19" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Accumulated Depreciation</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>All accumulated depreciation and amortization (enter as negative number)</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n"/>
+      <c r="C15" s="19" t="n"/>
     </row>
     <row r="16" ht="8" customHeight="1">
-      <c r="C16" s="2" t="n"/>
+      <c r="C16" s="13" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>OTHER ASSETS</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n"/>
+      <c r="C17" s="13" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Inter Company Receivable</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="18" t="inlineStr">
         <is>
           <t>All amounts owed by a related company</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
+      <c r="C18" s="19" t="n"/>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Other Assets</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="18" t="inlineStr">
         <is>
           <t>Hauling authorities, cash value life insurance, investment in other companies, condos, boats, long term owner receivables, etc.</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n"/>
+      <c r="C19" s="19" t="n"/>
     </row>
     <row r="20" ht="8" customHeight="1">
-      <c r="C20" s="2" t="n"/>
+      <c r="C20" s="13" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>CURRENT LIABILITIES</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n"/>
+      <c r="C21" s="13" t="n"/>
     </row>
     <row r="22" ht="30" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Bank</t>
         </is>
       </c>
-      <c r="B22" s="7" t="inlineStr">
+      <c r="B22" s="18" t="inlineStr">
         <is>
           <t>Bank revolving line of credit outstanding</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
+      <c r="C22" s="19" t="n"/>
     </row>
     <row r="23" ht="30" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Owners</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr"/>
-      <c r="C23" s="8" t="n"/>
+      <c r="B23" s="18" t="inlineStr"/>
+      <c r="C23" s="19" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Payable</t>
         </is>
       </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B24" s="18" t="inlineStr">
         <is>
           <t>Accounts payable to vendors, suppliers, other agents, etc.</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
+      <c r="C24" s="19" t="n"/>
     </row>
     <row r="25" ht="30" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Accrued Expenses</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B25" s="18" t="inlineStr">
         <is>
           <t>Salary, vacation pay, interest, etc.</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
+      <c r="C25" s="19" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Current Portion LTD</t>
         </is>
       </c>
-      <c r="B26" s="7" t="inlineStr">
+      <c r="B26" s="18" t="inlineStr">
         <is>
           <t>Current portion of interest bearing long term debt</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
+      <c r="C26" s="19" t="n"/>
     </row>
     <row r="27" ht="30" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Inter Company Payable</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>All amounts owed to a related company</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
+      <c r="C27" s="19" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1">
-      <c r="A28" s="6" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Other Current Liabilities</t>
         </is>
       </c>
-      <c r="B28" s="7" t="inlineStr">
+      <c r="B28" s="18" t="inlineStr">
         <is>
           <t>Deferred taxes, income tax payable, etc.</t>
         </is>
       </c>
-      <c r="C28" s="8" t="n"/>
+      <c r="C28" s="19" t="n"/>
     </row>
     <row r="29" ht="8" customHeight="1">
-      <c r="C29" s="2" t="n"/>
+      <c r="C29" s="13" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>LONG-TERM LIABILITIES</t>
         </is>
       </c>
-      <c r="C30" s="2" t="n"/>
+      <c r="C30" s="13" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>EID Loan</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr"/>
-      <c r="C31" s="8" t="n"/>
+      <c r="B31" s="18" t="inlineStr"/>
+      <c r="C31" s="19" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Long-term Debt</t>
         </is>
       </c>
-      <c r="B32" s="7" t="inlineStr">
+      <c r="B32" s="18" t="inlineStr">
         <is>
           <t>All interest bearing non-owner debt and non inter-company debt</t>
         </is>
       </c>
-      <c r="C32" s="8" t="n"/>
+      <c r="C32" s="19" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="6" t="inlineStr">
+      <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Notes Payable Owners (LT)</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="18" t="inlineStr">
         <is>
           <t>Amounts due to owners - long term</t>
         </is>
       </c>
-      <c r="C33" s="8" t="n"/>
+      <c r="C33" s="19" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+      <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Inter Company Debt</t>
         </is>
       </c>
-      <c r="B34" s="7" t="inlineStr">
+      <c r="B34" s="18" t="inlineStr">
         <is>
           <t>All amounts owed to a related company</t>
         </is>
       </c>
-      <c r="C34" s="8" t="n"/>
+      <c r="C34" s="19" t="n"/>
     </row>
     <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Other LT Liabilities</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="18" t="inlineStr">
         <is>
           <t>Life insurance loans, etc.</t>
         </is>
       </c>
-      <c r="C35" s="8" t="n"/>
+      <c r="C35" s="19" t="n"/>
     </row>
     <row r="36" ht="8" customHeight="1">
-      <c r="C36" s="2" t="n"/>
+      <c r="C36" s="13" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>EQUITY</t>
         </is>
       </c>
-      <c r="C37" s="2" t="n"/>
+      <c r="C37" s="13" t="n"/>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Owner's Equity</t>
         </is>
       </c>
-      <c r="B38" s="7" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>Assets minus liabilities (Net Worth)</t>
         </is>
       </c>
-      <c r="C38" s="8" t="n"/>
+      <c r="C38" s="19" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="7">
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A37:C37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Improve template readability and add numeric data validation
- Increased font sizes for line items (12pt bold) and descriptions (11pt)
- Added Excel data validation on Amount column to reject non-numeric input
- Number format allows up to 4 decimal places
- Renamed column header from "12/31/25" to "Amount"

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -19,9 +19,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,19 +61,37 @@
       <sz val="13"/>
     </font>
     <font>
+      <name val="Montserrat"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="16"/>
     </font>
     <font>
+      <name val="Montserrat"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Montserrat"/>
+      <color rgb="004a5568"/>
       <sz val="11"/>
     </font>
     <font>
-      <i val="1"/>
-      <color rgb="004a5568"/>
-      <sz val="9"/>
+      <name val="Montserrat"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -176,16 +194,16 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -881,7 +899,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Income Statement Data Entry</t>
@@ -889,7 +907,7 @@
       </c>
       <c r="C1" s="13" t="n"/>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Line Item</t>
@@ -902,11 +920,11 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>12/31/25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
         <is>
           <t>REVENUE</t>
@@ -914,7 +932,7 @@
       </c>
       <c r="C3" s="13" t="n"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Intra State HHG</t>
@@ -927,7 +945,7 @@
       </c>
       <c r="C4" s="19" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Local HHG</t>
@@ -940,7 +958,7 @@
       </c>
       <c r="C5" s="19" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Inter State HHG</t>
@@ -953,7 +971,7 @@
       </c>
       <c r="C6" s="19" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Office &amp; Industrial</t>
@@ -966,7 +984,7 @@
       </c>
       <c r="C7" s="19" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Warehouse (Non-commercial)</t>
@@ -979,7 +997,7 @@
       </c>
       <c r="C8" s="19" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Warehouse Handling (Non-commercial)</t>
@@ -988,7 +1006,7 @@
       <c r="B9" s="18" t="inlineStr"/>
       <c r="C9" s="19" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>International</t>
@@ -1001,7 +1019,7 @@
       </c>
       <c r="C10" s="19" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Packing &amp; Unpacking</t>
@@ -1014,7 +1032,7 @@
       </c>
       <c r="C11" s="19" t="n"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="32" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Booking &amp; Royalties</t>
@@ -1027,7 +1045,7 @@
       </c>
       <c r="C12" s="19" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1">
+    <row r="13" ht="32" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Special Products</t>
@@ -1040,7 +1058,7 @@
       </c>
       <c r="C13" s="19" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Records Storage</t>
@@ -1053,7 +1071,7 @@
       </c>
       <c r="C14" s="19" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Military DPM Contracts</t>
@@ -1066,7 +1084,7 @@
       </c>
       <c r="C15" s="19" t="n"/>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="32" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Distribution</t>
@@ -1079,7 +1097,7 @@
       </c>
       <c r="C16" s="19" t="n"/>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="32" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Hotel Deliveries</t>
@@ -1092,7 +1110,7 @@
       </c>
       <c r="C17" s="19" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Other Revenue</t>
@@ -1108,7 +1126,7 @@
     <row r="19" ht="8" customHeight="1">
       <c r="C19" s="13" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1">
+    <row r="20" ht="25" customHeight="1">
       <c r="A20" s="16" t="inlineStr">
         <is>
           <t>DIRECT EXPENSES (COST OF REVENUE)</t>
@@ -1116,7 +1134,7 @@
       </c>
       <c r="C20" s="13" t="n"/>
     </row>
-    <row r="21" ht="30" customHeight="1">
+    <row r="21" ht="32" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Direct Wages</t>
@@ -1129,7 +1147,7 @@
       </c>
       <c r="C21" s="19" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="32" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Vehicle Operating Expense</t>
@@ -1142,7 +1160,7 @@
       </c>
       <c r="C22" s="19" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="32" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Packing/Warehouse Supplies</t>
@@ -1155,7 +1173,7 @@
       </c>
       <c r="C23" s="19" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="32" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
           <t>OO Exp Intra State</t>
@@ -1168,7 +1186,7 @@
       </c>
       <c r="C24" s="19" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="32" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>OO Inter State</t>
@@ -1181,7 +1199,7 @@
       </c>
       <c r="C25" s="19" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="32" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
           <t>OO O&amp;I</t>
@@ -1194,7 +1212,7 @@
       </c>
       <c r="C26" s="19" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>OO Packing</t>
@@ -1207,7 +1225,7 @@
       </c>
       <c r="C27" s="19" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
           <t>OO Other</t>
@@ -1220,7 +1238,7 @@
       </c>
       <c r="C28" s="19" t="n"/>
     </row>
-    <row r="29" ht="30" customHeight="1">
+    <row r="29" ht="32" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Claims</t>
@@ -1233,7 +1251,7 @@
       </c>
       <c r="C29" s="19" t="n"/>
     </row>
-    <row r="30" ht="30" customHeight="1">
+    <row r="30" ht="32" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Other Trans Exp</t>
@@ -1246,7 +1264,7 @@
       </c>
       <c r="C30" s="19" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Depreciation</t>
@@ -1259,7 +1277,7 @@
       </c>
       <c r="C31" s="19" t="n"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Lease Expense Rev Equip</t>
@@ -1272,7 +1290,7 @@
       </c>
       <c r="C32" s="19" t="n"/>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Rent</t>
@@ -1285,7 +1303,7 @@
       </c>
       <c r="C33" s="19" t="n"/>
     </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Other Direct Expenses</t>
@@ -1301,7 +1319,7 @@
     <row r="35" ht="8" customHeight="1">
       <c r="C35" s="13" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="25" customHeight="1">
       <c r="A36" s="16" t="inlineStr">
         <is>
           <t>OPERATING EXPENSES</t>
@@ -1309,7 +1327,7 @@
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" ht="30" customHeight="1">
+    <row r="37" ht="32" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Advertising/Marketing</t>
@@ -1322,7 +1340,7 @@
       </c>
       <c r="C37" s="19" t="n"/>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Bad Debts</t>
@@ -1335,7 +1353,7 @@
       </c>
       <c r="C38" s="19" t="n"/>
     </row>
-    <row r="39" ht="30" customHeight="1">
+    <row r="39" ht="32" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Sales Commissions</t>
@@ -1348,7 +1366,7 @@
       </c>
       <c r="C39" s="19" t="n"/>
     </row>
-    <row r="40" ht="30" customHeight="1">
+    <row r="40" ht="32" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Contributions</t>
@@ -1357,7 +1375,7 @@
       <c r="B40" s="18" t="inlineStr"/>
       <c r="C40" s="19" t="n"/>
     </row>
-    <row r="41" ht="30" customHeight="1">
+    <row r="41" ht="32" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Computer Support</t>
@@ -1370,7 +1388,7 @@
       </c>
       <c r="C41" s="19" t="n"/>
     </row>
-    <row r="42" ht="30" customHeight="1">
+    <row r="42" ht="32" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Dues &amp; Subscriptions</t>
@@ -1379,7 +1397,7 @@
       <c r="B42" s="18" t="inlineStr"/>
       <c r="C42" s="19" t="n"/>
     </row>
-    <row r="43" ht="30" customHeight="1">
+    <row r="43" ht="32" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
           <t>PR Taxes &amp; Benefits</t>
@@ -1392,7 +1410,7 @@
       </c>
       <c r="C43" s="19" t="n"/>
     </row>
-    <row r="44" ht="30" customHeight="1">
+    <row r="44" ht="32" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Equipment Leases Office Equip</t>
@@ -1401,7 +1419,7 @@
       <c r="B44" s="18" t="inlineStr"/>
       <c r="C44" s="19" t="n"/>
     </row>
-    <row r="45" ht="30" customHeight="1">
+    <row r="45" ht="32" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Workman's Comp Insurance</t>
@@ -1410,7 +1428,7 @@
       <c r="B45" s="18" t="inlineStr"/>
       <c r="C45" s="19" t="n"/>
     </row>
-    <row r="46" ht="30" customHeight="1">
+    <row r="46" ht="32" customHeight="1">
       <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Insurance</t>
@@ -1423,7 +1441,7 @@
       </c>
       <c r="C46" s="19" t="n"/>
     </row>
-    <row r="47" ht="30" customHeight="1">
+    <row r="47" ht="32" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Legal &amp; Accounting</t>
@@ -1436,7 +1454,7 @@
       </c>
       <c r="C47" s="19" t="n"/>
     </row>
-    <row r="48" ht="30" customHeight="1">
+    <row r="48" ht="32" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Office Expense</t>
@@ -1449,7 +1467,7 @@
       </c>
       <c r="C48" s="19" t="n"/>
     </row>
-    <row r="49" ht="30" customHeight="1">
+    <row r="49" ht="32" customHeight="1">
       <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Other Admin</t>
@@ -1458,7 +1476,7 @@
       <c r="B49" s="18" t="inlineStr"/>
       <c r="C49" s="19" t="n"/>
     </row>
-    <row r="50" ht="30" customHeight="1">
+    <row r="50" ht="32" customHeight="1">
       <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Pension/Profit Sharing/401k</t>
@@ -1467,7 +1485,7 @@
       <c r="B50" s="18" t="inlineStr"/>
       <c r="C50" s="19" t="n"/>
     </row>
-    <row r="51" ht="30" customHeight="1">
+    <row r="51" ht="32" customHeight="1">
       <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Professional Fees</t>
@@ -1480,7 +1498,7 @@
       </c>
       <c r="C51" s="19" t="n"/>
     </row>
-    <row r="52" ht="30" customHeight="1">
+    <row r="52" ht="32" customHeight="1">
       <c r="A52" s="17" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
@@ -1489,7 +1507,7 @@
       <c r="B52" s="18" t="inlineStr"/>
       <c r="C52" s="19" t="n"/>
     </row>
-    <row r="53" ht="30" customHeight="1">
+    <row r="53" ht="32" customHeight="1">
       <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Salaries Admin</t>
@@ -1502,7 +1520,7 @@
       </c>
       <c r="C53" s="19" t="n"/>
     </row>
-    <row r="54" ht="30" customHeight="1">
+    <row r="54" ht="32" customHeight="1">
       <c r="A54" s="17" t="inlineStr">
         <is>
           <t>Taxes &amp; Licenses</t>
@@ -1515,7 +1533,7 @@
       </c>
       <c r="C54" s="19" t="n"/>
     </row>
-    <row r="55" ht="30" customHeight="1">
+    <row r="55" ht="32" customHeight="1">
       <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Tel/Fax/Utilities/Internet</t>
@@ -1528,7 +1546,7 @@
       </c>
       <c r="C55" s="19" t="n"/>
     </row>
-    <row r="56" ht="30" customHeight="1">
+    <row r="56" ht="32" customHeight="1">
       <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Travel &amp; Entertainment</t>
@@ -1541,7 +1559,7 @@
       </c>
       <c r="C56" s="19" t="n"/>
     </row>
-    <row r="57" ht="30" customHeight="1">
+    <row r="57" ht="32" customHeight="1">
       <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Vehicle Expense Admin</t>
@@ -1553,7 +1571,7 @@
     <row r="58" ht="8" customHeight="1">
       <c r="C58" s="13" t="n"/>
     </row>
-    <row r="59" ht="18" customHeight="1">
+    <row r="59" ht="25" customHeight="1">
       <c r="A59" s="16" t="inlineStr">
         <is>
           <t>OTHER INCOME/EXPENSES</t>
@@ -1561,7 +1579,7 @@
       </c>
       <c r="C59" s="13" t="n"/>
     </row>
-    <row r="60" ht="30" customHeight="1">
+    <row r="60" ht="32" customHeight="1">
       <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Other Income</t>
@@ -1574,7 +1592,7 @@
       </c>
       <c r="C60" s="19" t="n"/>
     </row>
-    <row r="61" ht="30" customHeight="1">
+    <row r="61" ht="32" customHeight="1">
       <c r="A61" s="17" t="inlineStr">
         <is>
           <t>CEO Comp</t>
@@ -1587,7 +1605,7 @@
       </c>
       <c r="C61" s="19" t="n"/>
     </row>
-    <row r="62" ht="30" customHeight="1">
+    <row r="62" ht="32" customHeight="1">
       <c r="A62" s="17" t="inlineStr">
         <is>
           <t>Other Expense</t>
@@ -1600,7 +1618,7 @@
       </c>
       <c r="C62" s="19" t="n"/>
     </row>
-    <row r="63" ht="30" customHeight="1">
+    <row r="63" ht="32" customHeight="1">
       <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Interest Expense</t>
@@ -1622,6 +1640,12 @@
     <mergeCell ref="A59:C59"/>
     <mergeCell ref="A20:C20"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
+      <formula1>-999999999999</formula1>
+      <formula2>999999999999</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1640,7 +1664,7 @@
     <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="25" customHeight="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Balance Sheet Data Entry</t>
@@ -1648,7 +1672,7 @@
       </c>
       <c r="C1" s="13" t="n"/>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Line Item</t>
@@ -1661,11 +1685,11 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
-          <t>12/31/25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
+          <t>Amount</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="25" customHeight="1">
       <c r="A3" s="16" t="inlineStr">
         <is>
           <t>CURRENT ASSETS</t>
@@ -1673,7 +1697,7 @@
       </c>
       <c r="C3" s="13" t="n"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="32" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Cash &amp; Cash Equivalents</t>
@@ -1686,7 +1710,7 @@
       </c>
       <c r="C4" s="19" t="n"/>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="32" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Receivable</t>
@@ -1699,7 +1723,7 @@
       </c>
       <c r="C5" s="19" t="n"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
+    <row r="6" ht="32" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Receivables</t>
@@ -1712,7 +1736,7 @@
       </c>
       <c r="C6" s="19" t="n"/>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="32" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Other Receivables</t>
@@ -1725,7 +1749,7 @@
       </c>
       <c r="C7" s="19" t="n"/>
     </row>
-    <row r="8" ht="30" customHeight="1">
+    <row r="8" ht="32" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Prepaid Expenses</t>
@@ -1738,7 +1762,7 @@
       </c>
       <c r="C8" s="19" t="n"/>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="32" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Related Company Receivables</t>
@@ -1751,7 +1775,7 @@
       </c>
       <c r="C9" s="19" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="32" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Owner Receivables</t>
@@ -1764,7 +1788,7 @@
       </c>
       <c r="C10" s="19" t="n"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="32" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Other Current Assets</t>
@@ -1780,7 +1804,7 @@
     <row r="12" ht="8" customHeight="1">
       <c r="C12" s="13" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
+    <row r="13" ht="25" customHeight="1">
       <c r="A13" s="16" t="inlineStr">
         <is>
           <t>FIXED ASSETS</t>
@@ -1788,7 +1812,7 @@
       </c>
       <c r="C13" s="13" t="n"/>
     </row>
-    <row r="14" ht="30" customHeight="1">
+    <row r="14" ht="32" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Gross Fixed Assets</t>
@@ -1801,7 +1825,7 @@
       </c>
       <c r="C14" s="19" t="n"/>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="32" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Accumulated Depreciation</t>
@@ -1817,7 +1841,7 @@
     <row r="16" ht="8" customHeight="1">
       <c r="C16" s="13" t="n"/>
     </row>
-    <row r="17" ht="18" customHeight="1">
+    <row r="17" ht="25" customHeight="1">
       <c r="A17" s="16" t="inlineStr">
         <is>
           <t>OTHER ASSETS</t>
@@ -1825,7 +1849,7 @@
       </c>
       <c r="C17" s="13" t="n"/>
     </row>
-    <row r="18" ht="30" customHeight="1">
+    <row r="18" ht="32" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Inter Company Receivable</t>
@@ -1838,7 +1862,7 @@
       </c>
       <c r="C18" s="19" t="n"/>
     </row>
-    <row r="19" ht="30" customHeight="1">
+    <row r="19" ht="32" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Other Assets</t>
@@ -1854,7 +1878,7 @@
     <row r="20" ht="8" customHeight="1">
       <c r="C20" s="13" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1">
+    <row r="21" ht="25" customHeight="1">
       <c r="A21" s="16" t="inlineStr">
         <is>
           <t>CURRENT LIABILITIES</t>
@@ -1862,7 +1886,7 @@
       </c>
       <c r="C21" s="13" t="n"/>
     </row>
-    <row r="22" ht="30" customHeight="1">
+    <row r="22" ht="32" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Bank</t>
@@ -1875,7 +1899,7 @@
       </c>
       <c r="C22" s="19" t="n"/>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="32" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Owners</t>
@@ -1884,7 +1908,7 @@
       <c r="B23" s="18" t="inlineStr"/>
       <c r="C23" s="19" t="n"/>
     </row>
-    <row r="24" ht="30" customHeight="1">
+    <row r="24" ht="32" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Payable</t>
@@ -1897,7 +1921,7 @@
       </c>
       <c r="C24" s="19" t="n"/>
     </row>
-    <row r="25" ht="30" customHeight="1">
+    <row r="25" ht="32" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Accrued Expenses</t>
@@ -1910,7 +1934,7 @@
       </c>
       <c r="C25" s="19" t="n"/>
     </row>
-    <row r="26" ht="30" customHeight="1">
+    <row r="26" ht="32" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Current Portion LTD</t>
@@ -1923,7 +1947,7 @@
       </c>
       <c r="C26" s="19" t="n"/>
     </row>
-    <row r="27" ht="30" customHeight="1">
+    <row r="27" ht="32" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Inter Company Payable</t>
@@ -1936,7 +1960,7 @@
       </c>
       <c r="C27" s="19" t="n"/>
     </row>
-    <row r="28" ht="30" customHeight="1">
+    <row r="28" ht="32" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Other Current Liabilities</t>
@@ -1952,7 +1976,7 @@
     <row r="29" ht="8" customHeight="1">
       <c r="C29" s="13" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1">
+    <row r="30" ht="25" customHeight="1">
       <c r="A30" s="16" t="inlineStr">
         <is>
           <t>LONG-TERM LIABILITIES</t>
@@ -1960,7 +1984,7 @@
       </c>
       <c r="C30" s="13" t="n"/>
     </row>
-    <row r="31" ht="30" customHeight="1">
+    <row r="31" ht="32" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>EID Loan</t>
@@ -1969,7 +1993,7 @@
       <c r="B31" s="18" t="inlineStr"/>
       <c r="C31" s="19" t="n"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="32" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Long-term Debt</t>
@@ -1982,7 +2006,7 @@
       </c>
       <c r="C32" s="19" t="n"/>
     </row>
-    <row r="33" ht="30" customHeight="1">
+    <row r="33" ht="32" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Notes Payable Owners (LT)</t>
@@ -1995,7 +2019,7 @@
       </c>
       <c r="C33" s="19" t="n"/>
     </row>
-    <row r="34" ht="30" customHeight="1">
+    <row r="34" ht="32" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Inter Company Debt</t>
@@ -2008,7 +2032,7 @@
       </c>
       <c r="C34" s="19" t="n"/>
     </row>
-    <row r="35" ht="30" customHeight="1">
+    <row r="35" ht="32" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Other LT Liabilities</t>
@@ -2024,7 +2048,7 @@
     <row r="36" ht="8" customHeight="1">
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="25" customHeight="1">
       <c r="A37" s="16" t="inlineStr">
         <is>
           <t>EQUITY</t>
@@ -2032,7 +2056,7 @@
       </c>
       <c r="C37" s="13" t="n"/>
     </row>
-    <row r="38" ht="30" customHeight="1">
+    <row r="38" ht="32" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Owner's Equity</t>
@@ -2056,6 +2080,12 @@
     <mergeCell ref="A21:C21"/>
     <mergeCell ref="A30:C30"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C14 C15 C18 C19 C22 C23 C24 C25 C26 C27 C28 C31 C32 C33 C34 C35 C38" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
+      <formula1>-999999999999</formula1>
+      <formula2>999999999999</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add administrative_employees field to upload workflow
Adds headcount input to the Income Statement form, Excel template,
and parser so the Revenue Per Admin Employee gauge can display
correct values. Computes rev_admin_employee on submit.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Income Statement" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Balance Sheet" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C63"/>
+  <dimension ref="A1:C66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1631,17 +1631,42 @@
       </c>
       <c r="C63" s="19" t="n"/>
     </row>
+    <row r="64" ht="8" customHeight="1">
+      <c r="C64" s="13" t="n"/>
+    </row>
+    <row r="65" ht="25" customHeight="1">
+      <c r="A65" s="16" t="inlineStr">
+        <is>
+          <t>LABOR ANALYSIS</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="n"/>
+    </row>
+    <row r="66" ht="32" customHeight="1">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Administrative Employees</t>
+        </is>
+      </c>
+      <c r="B66" s="18" t="inlineStr">
+        <is>
+          <t>Total number of admin employees (FTE). Include CEO, dispatch, office, managers, salaried sales. Exclude commissioned and hourly warehouse.</t>
+        </is>
+      </c>
+      <c r="C66" s="19" t="n"/>
+    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A65:C65"/>
     <mergeCell ref="A20:C20"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63 C66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
       <formula1>-999999999999</formula1>
       <formula2>999999999999</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add Number of Branches field to upload workflow and actuals display
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -891,7 +891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C66"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1654,6 +1654,19 @@
         </is>
       </c>
       <c r="C66" s="19" t="n"/>
+    </row>
+    <row r="67" ht="32" customHeight="1">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Number of Branches</t>
+        </is>
+      </c>
+      <c r="B67" s="18" t="inlineStr">
+        <is>
+          <t>Total number of branch locations operating under your company</t>
+        </is>
+      </c>
+      <c r="C67" s="19" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -1666,7 +1679,7 @@
     <mergeCell ref="A20:C20"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63 C66" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63 C66 C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
       <formula1>-999999999999</formula1>
       <formula2>999999999999</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Update line item descriptions from BPC template and improve Excel readability
- Fill in all missing descriptions from official BPC upload template
- Update existing descriptions with more detailed versions
- Widen description column and use dynamic row heights in Excel template
- Bump description font size for readability

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -87,7 +87,7 @@
     <font>
       <name val="Montserrat"/>
       <color rgb="004a5568"/>
-      <sz val="11"/>
+      <sz val="11.5"/>
     </font>
     <font>
       <name val="Montserrat"/>
@@ -895,7 +895,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -932,7 +932,7 @@
       </c>
       <c r="C3" s="13" t="n"/>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="56" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Intra State HHG</t>
@@ -940,12 +940,12 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Transportation revenues generated under an intrastate tariff</t>
+          <t>All transportation and accessorial revenues generated under an intrastate tariff (military, GSA, or civilian), or if no tariff, all revenues generated within your state, but not local</t>
         </is>
       </c>
       <c r="C4" s="19" t="n"/>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="40" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Local HHG</t>
@@ -953,12 +953,12 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Revenues defined by an intrastate tariff as local</t>
+          <t>All revenues defined by an intrastate tariff as local, or if no tariff, all revenues generated within the commercial zone of your city</t>
         </is>
       </c>
       <c r="C5" s="19" t="n"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Inter State HHG</t>
@@ -966,12 +966,12 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Transportation revenues generated under an interstate tariff</t>
+          <t>All transportation and accessorial revenues generated under an interstate tariff (military, GSA, or civilian)</t>
         </is>
       </c>
       <c r="C6" s="19" t="n"/>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="40" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Office &amp; Industrial</t>
@@ -979,12 +979,12 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>All local commercial revenue except HHG</t>
+          <t>All local commercial revenue except HHG and local distribution transportation</t>
         </is>
       </c>
       <c r="C7" s="19" t="n"/>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="40" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Warehouse (Non-commercial)</t>
@@ -992,21 +992,25 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>All permanent and SIT revenue</t>
+          <t>All permanent and SIT revenue, including delivery out of SIT, but excluding distribution revenues</t>
         </is>
       </c>
       <c r="C8" s="19" t="n"/>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Warehouse Handling (Non-commercial)</t>
         </is>
       </c>
-      <c r="B9" s="18" t="inlineStr"/>
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>All warehouse handling revenue</t>
+        </is>
+      </c>
       <c r="C9" s="19" t="n"/>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="40" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>International</t>
@@ -1014,12 +1018,12 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>All international revenue including pickup, packing, crating, delivery</t>
+          <t>All international revenue including pickup, packing, crating, delivery and accessorials; except for booking &amp; storage</t>
         </is>
       </c>
       <c r="C10" s="19" t="n"/>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Packing &amp; Unpacking</t>
@@ -1027,12 +1031,12 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>All revenue for packing, unpacking and container revenue</t>
+          <t>All revenue for packing, unpacking and container revenue for domestic HHG shipments</t>
         </is>
       </c>
       <c r="C11" s="19" t="n"/>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="40" customHeight="1">
       <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Booking &amp; Royalties</t>
@@ -1040,12 +1044,12 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Sales booking revenue and Operating Authority royalties</t>
+          <t>Sales booking revenue for all business lines &amp; Operating Authority royalties</t>
         </is>
       </c>
       <c r="C12" s="19" t="n"/>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="40" customHeight="1">
       <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Special Products</t>
@@ -1053,12 +1057,12 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>All special product revenue and HVP transportation</t>
+          <t>All special product revenue and HVP transportation, non HHG brokerage 3rd party, new lines of business</t>
         </is>
       </c>
       <c r="C13" s="19" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Records Storage</t>
@@ -1071,7 +1075,7 @@
       </c>
       <c r="C14" s="19" t="n"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Military DPM Contracts</t>
@@ -1079,12 +1083,12 @@
       </c>
       <c r="B15" s="18" t="inlineStr">
         <is>
-          <t>Revenues from Direct Procurement Method military contracts</t>
+          <t>All revenues from Direct Procurement Method military contracts, except storage revenues included in Warehouse above</t>
         </is>
       </c>
       <c r="C15" s="19" t="n"/>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16" ht="40" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Distribution</t>
@@ -1092,12 +1096,12 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>All distribution revenue</t>
+          <t>All distribution revenue, including commercial warehousing, logistics, kitting, hotel FFE projects, including handling</t>
         </is>
       </c>
       <c r="C16" s="19" t="n"/>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="28" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Hotel Deliveries</t>
@@ -1105,12 +1109,12 @@
       </c>
       <c r="B17" s="18" t="inlineStr">
         <is>
-          <t>All revenues from hotel deliveries</t>
+          <t>All revenues generated from hotel deliveries</t>
         </is>
       </c>
       <c r="C17" s="19" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="40" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Other Revenue</t>
@@ -1118,7 +1122,7 @@
       </c>
       <c r="B18" s="18" t="inlineStr">
         <is>
-          <t>Any misc. operational revenue not listed elsewhere</t>
+          <t>Any misc. operational revenue not listed elsewhere (ex. surveys, estimates, etc.)</t>
         </is>
       </c>
       <c r="C18" s="19" t="n"/>
@@ -1134,7 +1138,7 @@
       </c>
       <c r="C20" s="13" t="n"/>
     </row>
-    <row r="21" ht="32" customHeight="1">
+    <row r="21" ht="56" customHeight="1">
       <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Direct Wages</t>
@@ -1142,12 +1146,12 @@
       </c>
       <c r="B21" s="18" t="inlineStr">
         <is>
-          <t>Salaries, wages, and bonuses paid to operations personnel</t>
+          <t>All salaries, wages, and bonuses paid to operations personnel; including drivers, helpers, packers, warehousemen; excluding admin, office, dispatch and sales</t>
         </is>
       </c>
       <c r="C21" s="19" t="n"/>
     </row>
-    <row r="22" ht="32" customHeight="1">
+    <row r="22" ht="56" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Vehicle Operating Expense</t>
@@ -1155,12 +1159,12 @@
       </c>
       <c r="B22" s="18" t="inlineStr">
         <is>
-          <t>Repairs, fuel, license, registration, tires, permits for revenue equipment</t>
+          <t>All expenses for revenue equipment: repairs and maintenance, fuel, license, registration, tires/tubes, permits, painting, decaling, washing, etc.</t>
         </is>
       </c>
       <c r="C22" s="19" t="n"/>
     </row>
-    <row r="23" ht="32" customHeight="1">
+    <row r="23" ht="40" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Packing/Warehouse Supplies</t>
@@ -1168,12 +1172,12 @@
       </c>
       <c r="B23" s="18" t="inlineStr">
         <is>
-          <t>Moving and packing supplies</t>
+          <t>All moving and packing supplies, including cartons, newsprint, blankets, labels, liftvans, dollies, tools, and misc.</t>
         </is>
       </c>
       <c r="C23" s="19" t="n"/>
     </row>
-    <row r="24" ht="32" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
           <t>OO Exp Intra State</t>
@@ -1181,12 +1185,12 @@
       </c>
       <c r="B24" s="18" t="inlineStr">
         <is>
-          <t>Payments to owner operators for intrastate jobs</t>
+          <t>All payments to O/O for intrastate moves</t>
         </is>
       </c>
       <c r="C24" s="19" t="n"/>
     </row>
-    <row r="25" ht="32" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>OO Inter State</t>
@@ -1194,12 +1198,12 @@
       </c>
       <c r="B25" s="18" t="inlineStr">
         <is>
-          <t>Payments to owner operators for interstate jobs</t>
+          <t>All payments to O/O for interstate moves</t>
         </is>
       </c>
       <c r="C25" s="19" t="n"/>
     </row>
-    <row r="26" ht="32" customHeight="1">
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
           <t>OO O&amp;I</t>
@@ -1207,12 +1211,12 @@
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Payments to owner operators for office &amp; industrial jobs</t>
+          <t>All payments to O/O for O/I</t>
         </is>
       </c>
       <c r="C26" s="19" t="n"/>
     </row>
-    <row r="27" ht="32" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>OO Packing</t>
@@ -1220,12 +1224,12 @@
       </c>
       <c r="B27" s="18" t="inlineStr">
         <is>
-          <t>Payments to owner operators for packing jobs</t>
+          <t>All payments to O/O for packing/unpacking</t>
         </is>
       </c>
       <c r="C27" s="19" t="n"/>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28" ht="40" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
           <t>OO Other</t>
@@ -1233,12 +1237,12 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>Payments to owner operators for other job types</t>
+          <t>All payments to O/O for other work (if you do not track O/O expenses by type, put all O/O expenses here)</t>
         </is>
       </c>
       <c r="C28" s="19" t="n"/>
     </row>
-    <row r="29" ht="32" customHeight="1">
+    <row r="29" ht="28" customHeight="1">
       <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Claims</t>
@@ -1251,7 +1255,7 @@
       </c>
       <c r="C29" s="19" t="n"/>
     </row>
-    <row r="30" ht="32" customHeight="1">
+    <row r="30" ht="40" customHeight="1">
       <c r="A30" s="17" t="inlineStr">
         <is>
           <t>Other Trans Exp</t>
@@ -1259,12 +1263,12 @@
       </c>
       <c r="B30" s="18" t="inlineStr">
         <is>
-          <t>Trip expense, deadhead miles, agent fees, freight, BIPD</t>
+          <t>Trip expense, deadhead miles, agent fees, PUC, freight, BIPD, O/O physical damage insurance, employee per diems</t>
         </is>
       </c>
       <c r="C30" s="19" t="n"/>
     </row>
-    <row r="31" ht="32" customHeight="1">
+    <row r="31" ht="56" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>Depreciation</t>
@@ -1272,12 +1276,12 @@
       </c>
       <c r="B31" s="18" t="inlineStr">
         <is>
-          <t>Depreciation on assets (excluding buildings)</t>
+          <t>All depreciation and amortization of intangible assets, vehicles, revenue equipment, office furniture, fixtures, equipment, computer hardware &amp; software; excluding depreciation on buildings or leasehold improvements</t>
         </is>
       </c>
       <c r="C31" s="19" t="n"/>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Lease Expense Rev Equip</t>
@@ -1285,12 +1289,12 @@
       </c>
       <c r="B32" s="18" t="inlineStr">
         <is>
-          <t>All lease expense on revenue equipment</t>
+          <t>All lease expense on any revenue equipment</t>
         </is>
       </c>
       <c r="C32" s="19" t="n"/>
     </row>
-    <row r="33" ht="32" customHeight="1">
+    <row r="33" ht="56" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Rent</t>
@@ -1298,12 +1302,12 @@
       </c>
       <c r="B33" s="18" t="inlineStr">
         <is>
-          <t>Actual or estimated fair market rent</t>
+          <t>Actual rent/lease expenses if paid to an unrelated third party, or estimated Fair Market Rent on a triple net basis if building is owned by the company or a related party</t>
         </is>
       </c>
       <c r="C33" s="19" t="n"/>
     </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="34" ht="56" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Other Direct Expenses</t>
@@ -1311,7 +1315,7 @@
       </c>
       <c r="B34" s="18" t="inlineStr">
         <is>
-          <t>Credit card fees and other direct expenses not otherwise classified</t>
+          <t>Credit card fees and all other direct expenses not otherwise classified (uniforms, CBS charges, meals, laundry, tolls, delivery service, parking, etc.)</t>
         </is>
       </c>
       <c r="C34" s="19" t="n"/>
@@ -1327,7 +1331,7 @@
       </c>
       <c r="C36" s="13" t="n"/>
     </row>
-    <row r="37" ht="32" customHeight="1">
+    <row r="37" ht="40" customHeight="1">
       <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Advertising/Marketing</t>
@@ -1335,12 +1339,12 @@
       </c>
       <c r="B37" s="18" t="inlineStr">
         <is>
-          <t>Advertising, brochures, yellow pages, promotional items</t>
+          <t>All advertising and marketing expense, brochures, yellow pages, promotional items, telemarketing, web page expense, etc.</t>
         </is>
       </c>
       <c r="C37" s="19" t="n"/>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38" ht="40" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Bad Debts</t>
@@ -1348,12 +1352,12 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Uncollectible accounts receivable written off</t>
+          <t>Uncollectible accounts receivable written off and offsetting entries for Allowance for Doubtful Accounts</t>
         </is>
       </c>
       <c r="C38" s="19" t="n"/>
     </row>
-    <row r="39" ht="32" customHeight="1">
+    <row r="39" ht="40" customHeight="1">
       <c r="A39" s="17" t="inlineStr">
         <is>
           <t>Sales Commissions</t>
@@ -1361,21 +1365,25 @@
       </c>
       <c r="B39" s="18" t="inlineStr">
         <is>
-          <t>Salaries, commissions, and draws for sales people</t>
+          <t>All salaries, wages, and bonuses paid to sales people, including commissions &amp; draws (not including sales support people)</t>
         </is>
       </c>
       <c r="C39" s="19" t="n"/>
     </row>
-    <row r="40" ht="32" customHeight="1">
+    <row r="40" ht="28" customHeight="1">
       <c r="A40" s="17" t="inlineStr">
         <is>
           <t>Contributions</t>
         </is>
       </c>
-      <c r="B40" s="18" t="inlineStr"/>
+      <c r="B40" s="18" t="inlineStr">
+        <is>
+          <t>All charitable donations</t>
+        </is>
+      </c>
       <c r="C40" s="19" t="n"/>
     </row>
-    <row r="41" ht="32" customHeight="1">
+    <row r="41" ht="56" customHeight="1">
       <c r="A41" s="17" t="inlineStr">
         <is>
           <t>Computer Support</t>
@@ -1383,21 +1391,25 @@
       </c>
       <c r="B41" s="18" t="inlineStr">
         <is>
-          <t>IT expenses, software licensing, satellite tracking</t>
+          <t>All IT expenses, including computer &amp; networking support, consultants, software licensing/maintenance, service agreements, training, satellite tracking</t>
         </is>
       </c>
       <c r="C41" s="19" t="n"/>
     </row>
-    <row r="42" ht="32" customHeight="1">
+    <row r="42" ht="28" customHeight="1">
       <c r="A42" s="17" t="inlineStr">
         <is>
           <t>Dues &amp; Subscriptions</t>
         </is>
       </c>
-      <c r="B42" s="18" t="inlineStr"/>
+      <c r="B42" s="18" t="inlineStr">
+        <is>
+          <t>All club dues, organization dues and publication subscriptions</t>
+        </is>
+      </c>
       <c r="C42" s="19" t="n"/>
     </row>
-    <row r="43" ht="32" customHeight="1">
+    <row r="43" ht="56" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
         <is>
           <t>PR Taxes &amp; Benefits</t>
@@ -1405,30 +1417,38 @@
       </c>
       <c r="B43" s="18" t="inlineStr">
         <is>
-          <t>Payroll taxes, health insurance, drug testing, DOT physicals, training</t>
+          <t>All payroll taxes; life and health insurance; drug testing; MVR reports; background checks; DOT physicals; employee recognition &amp; awards; training; recruiting; convention expenses</t>
         </is>
       </c>
       <c r="C43" s="19" t="n"/>
     </row>
-    <row r="44" ht="32" customHeight="1">
+    <row r="44" ht="40" customHeight="1">
       <c r="A44" s="17" t="inlineStr">
         <is>
           <t>Equipment Leases Office Equip</t>
         </is>
       </c>
-      <c r="B44" s="18" t="inlineStr"/>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>All non-revenue equipment leases such as copy machines, computers, etc.</t>
+        </is>
+      </c>
       <c r="C44" s="19" t="n"/>
     </row>
-    <row r="45" ht="32" customHeight="1">
+    <row r="45" ht="28" customHeight="1">
       <c r="A45" s="17" t="inlineStr">
         <is>
           <t>Workman's Comp Insurance</t>
         </is>
       </c>
-      <c r="B45" s="18" t="inlineStr"/>
+      <c r="B45" s="18" t="inlineStr">
+        <is>
+          <t>Insurance premiums for workmen's comp</t>
+        </is>
+      </c>
       <c r="C45" s="19" t="n"/>
     </row>
-    <row r="46" ht="32" customHeight="1">
+    <row r="46" ht="40" customHeight="1">
       <c r="A46" s="17" t="inlineStr">
         <is>
           <t>Insurance</t>
@@ -1436,12 +1456,12 @@
       </c>
       <c r="B46" s="18" t="inlineStr">
         <is>
-          <t>Cargo, fleet, general liability insurance</t>
+          <t>All cargo, fleet, general liability and insurance not otherwise classified</t>
         </is>
       </c>
       <c r="C46" s="19" t="n"/>
     </row>
-    <row r="47" ht="32" customHeight="1">
+    <row r="47" ht="40" customHeight="1">
       <c r="A47" s="17" t="inlineStr">
         <is>
           <t>Legal &amp; Accounting</t>
@@ -1449,12 +1469,12 @@
       </c>
       <c r="B47" s="18" t="inlineStr">
         <is>
-          <t>Legal and accounting work, tax return preparation</t>
+          <t>Expenses for legal and accounting work, preparation of tax returns, financial statements, etc.</t>
         </is>
       </c>
       <c r="C47" s="19" t="n"/>
     </row>
-    <row r="48" ht="32" customHeight="1">
+    <row r="48" ht="40" customHeight="1">
       <c r="A48" s="17" t="inlineStr">
         <is>
           <t>Office Expense</t>
@@ -1462,30 +1482,38 @@
       </c>
       <c r="B48" s="18" t="inlineStr">
         <is>
-          <t>Office &amp; printer supplies, printed forms, coffee, janitorial</t>
+          <t>Office &amp; printer supplies; printed forms; coffee, sundries; janitorial; alarm, security &amp; camera systems; postage; FedEx; etc.</t>
         </is>
       </c>
       <c r="C48" s="19" t="n"/>
     </row>
-    <row r="49" ht="32" customHeight="1">
+    <row r="49" ht="40" customHeight="1">
       <c r="A49" s="17" t="inlineStr">
         <is>
           <t>Other Admin</t>
         </is>
       </c>
-      <c r="B49" s="18" t="inlineStr"/>
+      <c r="B49" s="18" t="inlineStr">
+        <is>
+          <t>All expenses not otherwise classified such as bank charges, payroll processing, credit checks, PowerTrack fees, other fees</t>
+        </is>
+      </c>
       <c r="C49" s="19" t="n"/>
     </row>
-    <row r="50" ht="32" customHeight="1">
+    <row r="50" ht="40" customHeight="1">
       <c r="A50" s="17" t="inlineStr">
         <is>
           <t>Pension/Profit Sharing/401k</t>
         </is>
       </c>
-      <c r="B50" s="18" t="inlineStr"/>
+      <c r="B50" s="18" t="inlineStr">
+        <is>
+          <t>Company contributions &amp; administrative costs of pension, profit sharing and 401k plans</t>
+        </is>
+      </c>
       <c r="C50" s="19" t="n"/>
     </row>
-    <row r="51" ht="32" customHeight="1">
+    <row r="51" ht="40" customHeight="1">
       <c r="A51" s="17" t="inlineStr">
         <is>
           <t>Professional Fees</t>
@@ -1493,21 +1521,25 @@
       </c>
       <c r="B51" s="18" t="inlineStr">
         <is>
-          <t>Consultants, detectives, non-trade professionals</t>
+          <t>All fees paid to consultants, detectives, non-trade professionals; does not include legal, accounting, or computer professionals</t>
         </is>
       </c>
       <c r="C51" s="19" t="n"/>
     </row>
-    <row r="52" ht="32" customHeight="1">
+    <row r="52" ht="40" customHeight="1">
       <c r="A52" s="17" t="inlineStr">
         <is>
           <t>Repairs &amp; Maintenance</t>
         </is>
       </c>
-      <c r="B52" s="18" t="inlineStr"/>
+      <c r="B52" s="18" t="inlineStr">
+        <is>
+          <t>All repairs &amp; maintenance for warehouses, offices &amp; office equipment, other vehicles &amp; equipment not included in Vehicle Operating Expense</t>
+        </is>
+      </c>
       <c r="C52" s="19" t="n"/>
     </row>
-    <row r="53" ht="32" customHeight="1">
+    <row r="53" ht="56" customHeight="1">
       <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Salaries Admin</t>
@@ -1515,12 +1547,12 @@
       </c>
       <c r="B53" s="18" t="inlineStr">
         <is>
-          <t>All non-operations salaries (admin, office, dispatch, sales support)</t>
+          <t>All salaries, wages, and bonuses paid to non-operations personnel; including admin, office, dispatch, sales support; excluding CEO compensation and sales compensation</t>
         </is>
       </c>
       <c r="C53" s="19" t="n"/>
     </row>
-    <row r="54" ht="32" customHeight="1">
+    <row r="54" ht="56" customHeight="1">
       <c r="A54" s="17" t="inlineStr">
         <is>
           <t>Taxes &amp; Licenses</t>
@@ -1528,12 +1560,12 @@
       </c>
       <c r="B54" s="18" t="inlineStr">
         <is>
-          <t>All taxes and licenses not related to vehicles or income</t>
+          <t>All taxes and licenses NOT related to vehicles, income tax, or real estate taxes (examples: personal property, intangible, city/county/state business licenses, franchise)</t>
         </is>
       </c>
       <c r="C54" s="19" t="n"/>
     </row>
-    <row r="55" ht="32" customHeight="1">
+    <row r="55" ht="40" customHeight="1">
       <c r="A55" s="17" t="inlineStr">
         <is>
           <t>Tel/Fax/Utilities/Internet</t>
@@ -1541,12 +1573,12 @@
       </c>
       <c r="B55" s="18" t="inlineStr">
         <is>
-          <t>All communication and utility expenses</t>
+          <t>All expenses for telephone, cellular phones, internet connectivity, radios, heat, water, lights, gas, garbage, etc.</t>
         </is>
       </c>
       <c r="C55" s="19" t="n"/>
     </row>
-    <row r="56" ht="32" customHeight="1">
+    <row r="56" ht="40" customHeight="1">
       <c r="A56" s="17" t="inlineStr">
         <is>
           <t>Travel &amp; Entertainment</t>
@@ -1554,18 +1586,22 @@
       </c>
       <c r="B56" s="18" t="inlineStr">
         <is>
-          <t>Admin/sales related transportation, meals, lodging</t>
+          <t>All admin or sales related transportation, meals, lodging, vehicle rental; excludes seminar &amp; convention fees</t>
         </is>
       </c>
       <c r="C56" s="19" t="n"/>
     </row>
-    <row r="57" ht="32" customHeight="1">
+    <row r="57" ht="40" customHeight="1">
       <c r="A57" s="17" t="inlineStr">
         <is>
           <t>Vehicle Expense Admin</t>
         </is>
       </c>
-      <c r="B57" s="18" t="inlineStr"/>
+      <c r="B57" s="18" t="inlineStr">
+        <is>
+          <t>All expenses for sales &amp; admin vehicles: repairs and maintenance, fuel, license, registration, tires/tubes, etc.</t>
+        </is>
+      </c>
       <c r="C57" s="19" t="n"/>
     </row>
     <row r="58" ht="8" customHeight="1">
@@ -1579,7 +1615,7 @@
       </c>
       <c r="C59" s="13" t="n"/>
     </row>
-    <row r="60" ht="32" customHeight="1">
+    <row r="60" ht="56" customHeight="1">
       <c r="A60" s="17" t="inlineStr">
         <is>
           <t>Other Income</t>
@@ -1587,12 +1623,12 @@
       </c>
       <c r="B60" s="18" t="inlineStr">
         <is>
-          <t>Interest income, gain on sale of asset, litigation income</t>
+          <t>All non-operational income such as interest income, gain on sale of asset, litigation income (forgiven PPP money, employee retention tax credits)</t>
         </is>
       </c>
       <c r="C60" s="19" t="n"/>
     </row>
-    <row r="61" ht="32" customHeight="1">
+    <row r="61" ht="40" customHeight="1">
       <c r="A61" s="17" t="inlineStr">
         <is>
           <t>CEO Comp</t>
@@ -1600,12 +1636,12 @@
       </c>
       <c r="B61" s="18" t="inlineStr">
         <is>
-          <t>All salaries, bonuses or perks paid to CEO (enter as negative)</t>
+          <t>All salaries, bonuses or perks paid to CEO (not all owners). Enter as a negative number</t>
         </is>
       </c>
       <c r="C61" s="19" t="n"/>
     </row>
-    <row r="62" ht="32" customHeight="1">
+    <row r="62" ht="56" customHeight="1">
       <c r="A62" s="17" t="inlineStr">
         <is>
           <t>Other Expense</t>
@@ -1613,12 +1649,12 @@
       </c>
       <c r="B62" s="18" t="inlineStr">
         <is>
-          <t>Loss on sale of asset, research of new business lines (enter as negative)</t>
+          <t>All non-operational expenses such as loss on sale of asset, research of new lines of business, including depreciation on building over Fair Market Rent. Enter as a negative number</t>
         </is>
       </c>
       <c r="C62" s="19" t="n"/>
     </row>
-    <row r="63" ht="32" customHeight="1">
+    <row r="63" ht="40" customHeight="1">
       <c r="A63" s="17" t="inlineStr">
         <is>
           <t>Interest Expense</t>
@@ -1626,7 +1662,7 @@
       </c>
       <c r="B63" s="18" t="inlineStr">
         <is>
-          <t>All interest paid on interest bearing debt (enter as negative)</t>
+          <t>All interest paid on interest bearing debt owed. Enter as a negative number</t>
         </is>
       </c>
       <c r="C63" s="19" t="n"/>
@@ -1642,7 +1678,7 @@
       </c>
       <c r="C65" s="13" t="n"/>
     </row>
-    <row r="66" ht="32" customHeight="1">
+    <row r="66" ht="56" customHeight="1">
       <c r="A66" s="17" t="inlineStr">
         <is>
           <t>Administrative Employees</t>
@@ -1650,12 +1686,12 @@
       </c>
       <c r="B66" s="18" t="inlineStr">
         <is>
-          <t>Admin employee headcount (FTE): CEO, dispatch, office, managers, salaried sales</t>
+          <t>Admin employee headcount (FTE). Include: CEO, dispatch, office workers, managers, salaried sales. Exclude: commissioned employees, hourly warehouse employees. Use decimals for part-time</t>
         </is>
       </c>
       <c r="C66" s="19" t="n"/>
     </row>
-    <row r="67" ht="32" customHeight="1">
+    <row r="67" ht="56" customHeight="1">
       <c r="A67" s="17" t="inlineStr">
         <is>
           <t>Number of Branches</t>
@@ -1663,7 +1699,7 @@
       </c>
       <c r="B67" s="18" t="inlineStr">
         <is>
-          <t>Total number of branch locations operating under your company</t>
+          <t>Count of locations/branches with admin staff. Include: multiple office branches in different or same cities. Exclude: warehouses without admin staff</t>
         </is>
       </c>
       <c r="C67" s="19" t="n"/>
@@ -1698,7 +1734,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1735,7 +1771,7 @@
       </c>
       <c r="C3" s="13" t="n"/>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Cash &amp; Cash Equivalents</t>
@@ -1748,7 +1784,7 @@
       </c>
       <c r="C4" s="19" t="n"/>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Receivable</t>
@@ -1756,12 +1792,12 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Receivables generated from customers in the course of business</t>
+          <t>All receivables generated in the course of business from customers</t>
         </is>
       </c>
       <c r="C5" s="19" t="n"/>
     </row>
-    <row r="6" ht="32" customHeight="1">
+    <row r="6" ht="40" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Receivables</t>
@@ -1774,7 +1810,7 @@
       </c>
       <c r="C6" s="19" t="n"/>
     </row>
-    <row r="7" ht="32" customHeight="1">
+    <row r="7" ht="28" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Other Receivables</t>
@@ -1782,12 +1818,12 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Amounts owed by drivers, employees, etc.</t>
+          <t>All other receivables such as drivers, employees, etc.</t>
         </is>
       </c>
       <c r="C7" s="19" t="n"/>
     </row>
-    <row r="8" ht="32" customHeight="1">
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Prepaid Expenses</t>
@@ -1800,7 +1836,7 @@
       </c>
       <c r="C8" s="19" t="n"/>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="28" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Related Company Receivables</t>
@@ -1813,7 +1849,7 @@
       </c>
       <c r="C9" s="19" t="n"/>
     </row>
-    <row r="10" ht="32" customHeight="1">
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Owner Receivables</t>
@@ -1826,7 +1862,7 @@
       </c>
       <c r="C10" s="19" t="n"/>
     </row>
-    <row r="11" ht="32" customHeight="1">
+    <row r="11" ht="40" customHeight="1">
       <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Other Current Assets</t>
@@ -1834,7 +1870,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Packing supplies, investments not included in cash, etc.</t>
+          <t>All other current assets, such as packing supplies and investments not included in cash above</t>
         </is>
       </c>
       <c r="C11" s="19" t="n"/>
@@ -1850,7 +1886,7 @@
       </c>
       <c r="C13" s="13" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="40" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Gross Fixed Assets</t>
@@ -1863,7 +1899,7 @@
       </c>
       <c r="C14" s="19" t="n"/>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="40" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Accumulated Depreciation</t>
@@ -1887,7 +1923,7 @@
       </c>
       <c r="C17" s="13" t="n"/>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Inter Company Receivable</t>
@@ -1900,7 +1936,7 @@
       </c>
       <c r="C18" s="19" t="n"/>
     </row>
-    <row r="19" ht="32" customHeight="1">
+    <row r="19" ht="56" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Other Assets</t>
@@ -1908,7 +1944,7 @@
       </c>
       <c r="B19" s="18" t="inlineStr">
         <is>
-          <t>Hauling authorities, cash value life insurance, investment in other companies, condos, boats, long term owner receivables, etc.</t>
+          <t>All other assets such as hauling authorities, cash value life insurance, investment in other companies, condos, boats, long term owner receivables, etc.</t>
         </is>
       </c>
       <c r="C19" s="19" t="n"/>
@@ -1924,7 +1960,7 @@
       </c>
       <c r="C21" s="13" t="n"/>
     </row>
-    <row r="22" ht="32" customHeight="1">
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Bank</t>
@@ -1937,16 +1973,20 @@
       </c>
       <c r="C22" s="19" t="n"/>
     </row>
-    <row r="23" ht="32" customHeight="1">
+    <row r="23" ht="28" customHeight="1">
       <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Notes Payable/Owners</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr"/>
+      <c r="B23" s="18" t="inlineStr">
+        <is>
+          <t>Current portion of notes payable to owners</t>
+        </is>
+      </c>
       <c r="C23" s="19" t="n"/>
     </row>
-    <row r="24" ht="32" customHeight="1">
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Trade Accounts Payable</t>
@@ -1959,7 +1999,7 @@
       </c>
       <c r="C24" s="19" t="n"/>
     </row>
-    <row r="25" ht="32" customHeight="1">
+    <row r="25" ht="28" customHeight="1">
       <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Accrued Expenses</t>
@@ -1972,7 +2012,7 @@
       </c>
       <c r="C25" s="19" t="n"/>
     </row>
-    <row r="26" ht="32" customHeight="1">
+    <row r="26" ht="40" customHeight="1">
       <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Current Portion LTD</t>
@@ -1980,12 +2020,12 @@
       </c>
       <c r="B26" s="18" t="inlineStr">
         <is>
-          <t>Current portion of interest bearing long term debt</t>
+          <t>Current portion of interest bearing long term debt, excluding related company and owner debt</t>
         </is>
       </c>
       <c r="C26" s="19" t="n"/>
     </row>
-    <row r="27" ht="32" customHeight="1">
+    <row r="27" ht="28" customHeight="1">
       <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Inter Company Payable</t>
@@ -1998,7 +2038,7 @@
       </c>
       <c r="C27" s="19" t="n"/>
     </row>
-    <row r="28" ht="32" customHeight="1">
+    <row r="28" ht="40" customHeight="1">
       <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Other Current Liabilities</t>
@@ -2006,7 +2046,7 @@
       </c>
       <c r="B28" s="18" t="inlineStr">
         <is>
-          <t>Deferred taxes, income tax payable, etc.</t>
+          <t>All other current liabilities such as deferred taxes, income tax payable, etc.</t>
         </is>
       </c>
       <c r="C28" s="19" t="n"/>
@@ -2022,16 +2062,20 @@
       </c>
       <c r="C30" s="13" t="n"/>
     </row>
-    <row r="31" ht="32" customHeight="1">
+    <row r="31" ht="28" customHeight="1">
       <c r="A31" s="17" t="inlineStr">
         <is>
           <t>EID Loan</t>
         </is>
       </c>
-      <c r="B31" s="18" t="inlineStr"/>
+      <c r="B31" s="18" t="inlineStr">
+        <is>
+          <t>Amounts due on EIDL and/or PPP Loans (not forgiven)</t>
+        </is>
+      </c>
       <c r="C31" s="19" t="n"/>
     </row>
-    <row r="32" ht="32" customHeight="1">
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Long-term Debt</t>
@@ -2044,7 +2088,7 @@
       </c>
       <c r="C32" s="19" t="n"/>
     </row>
-    <row r="33" ht="32" customHeight="1">
+    <row r="33" ht="28" customHeight="1">
       <c r="A33" s="17" t="inlineStr">
         <is>
           <t>Notes Payable Owners (LT)</t>
@@ -2057,7 +2101,7 @@
       </c>
       <c r="C33" s="19" t="n"/>
     </row>
-    <row r="34" ht="32" customHeight="1">
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>Inter Company Debt</t>
@@ -2070,7 +2114,7 @@
       </c>
       <c r="C34" s="19" t="n"/>
     </row>
-    <row r="35" ht="32" customHeight="1">
+    <row r="35" ht="28" customHeight="1">
       <c r="A35" s="17" t="inlineStr">
         <is>
           <t>Other LT Liabilities</t>
@@ -2078,7 +2122,7 @@
       </c>
       <c r="B35" s="18" t="inlineStr">
         <is>
-          <t>Life insurance loans, etc.</t>
+          <t>All other long term liabilities such as life insurance loans, etc.</t>
         </is>
       </c>
       <c r="C35" s="19" t="n"/>
@@ -2094,7 +2138,7 @@
       </c>
       <c r="C37" s="13" t="n"/>
     </row>
-    <row r="38" ht="32" customHeight="1">
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Owner's Equity</t>
@@ -2102,7 +2146,7 @@
       </c>
       <c r="B38" s="18" t="inlineStr">
         <is>
-          <t>Assets minus liabilities (Net Worth)</t>
+          <t>Assets minus liabilities</t>
         </is>
       </c>
       <c r="C38" s="19" t="n"/>

</xml_diff>

<commit_message>
Fix upload template to display large numbers and remove digit limits
Widen amount column from 15 to 22, change number format from #,##0.0000
to #,##0, and remove range validation so any size number is accepted
while still rejecting text and special characters.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_Upload_Template.xlsx
@@ -18,9 +18,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0.0000"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="12">
     <font>
       <name val="Calibri"/>
@@ -203,7 +201,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
@@ -896,7 +894,7 @@
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -1715,10 +1713,7 @@
     <mergeCell ref="A20:C20"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63 C66 C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
-      <formula1>-999999999999</formula1>
-      <formula2>999999999999</formula2>
-    </dataValidation>
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C21 C22 C23 C24 C25 C26 C27 C28 C29 C30 C31 C32 C33 C34 C37 C38 C39 C40 C41 C42 C43 C44 C45 C46 C47 C48 C49 C50 C51 C52 C53 C54 C55 C56 C57 C60 C61 C62 C63 C66 C67" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1735,7 +1730,7 @@
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
     <col width="75" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="35" customHeight="1">
@@ -2163,10 +2158,7 @@
     <mergeCell ref="A30:C30"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C14 C15 C18 C19 C22 C23 C24 C25 C26 C27 C28 C31 C32 C33 C34 C35 C38" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal" operator="between">
-      <formula1>-999999999999</formula1>
-      <formula2>999999999999</formula2>
-    </dataValidation>
+    <dataValidation sqref="C4 C5 C6 C7 C8 C9 C10 C11 C14 C15 C18 C19 C22 C23 C24 C25 C26 C27 C28 C31 C32 C33 C34 C35 C38" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Invalid Entry" error="Please enter a number only. No dollar signs, commas, or text." promptTitle="Amount" prompt="Enter the dollar amount as a number (e.g., 150000 or -5000)" type="decimal"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>